<commit_message>
Fixed BOM and symbols on readme
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dario\Documents\NFC-lock-box\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C0EE48-0ECF-4885-AFDC-CCBE98A8C81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A90232-2AE3-49EB-BEDE-AA924D865170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{684F5010-FC7E-4A28-91AC-5FD8EFA55435}"/>
   </bookViews>
@@ -916,8 +916,8 @@
         <v>9</v>
       </c>
       <c r="C15">
-        <f>SUM(C2:C13)</f>
-        <v>41.830000000000005</v>
+        <f>SUM(C2:C14)</f>
+        <v>47.970000000000006</v>
       </c>
       <c r="D15" t="s">
         <v>20</v>

</xml_diff>